<commit_message>
Correocion a logica de guardado
</commit_message>
<xml_diff>
--- a/Base para el como vamos.xlsx
+++ b/Base para el como vamos.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG21"/>
+  <dimension ref="A1:AG19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -586,7 +586,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B2" t="n">
         <v>700000003</v>
@@ -610,7 +610,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>9175</v>
+        <v>0</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
@@ -655,7 +655,7 @@
         <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W2" t="n">
         <v>0</v>
@@ -699,7 +699,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B3" t="n">
         <v>700000003</v>
@@ -718,20 +718,12 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1694138</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>YENNY COROMOTO DIAZ PEREZ</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>9640</v>
+        <v>9376</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -740,21 +732,21 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>$504636.00</t>
+          <t>$000.00</t>
         </is>
       </c>
       <c r="L3" t="n">
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>3.45%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P3" t="n">
@@ -764,43 +756,43 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z3" t="n">
         <v>0</v>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="AB3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="AD3" t="n">
@@ -810,17 +802,17 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>$5677.16</t>
+          <t>$000.00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B4" t="n">
         <v>700000003</v>
@@ -839,39 +831,43 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1099653</v>
+        <v>1297183</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ANGELA MIREYA MONTENEGRO ROMERO</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>DORA INES BELTRAN GAMBA</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I4" t="n">
-        <v>9334</v>
+        <v>9948</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>$42028948.63</t>
+          <t>$000.00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>$7803091.00</t>
+          <t>$5178045.00</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>18.57</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>19.79%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P4" t="n">
@@ -881,63 +877,63 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>-11</v>
+        <v>3</v>
       </c>
       <c r="S4" t="n">
-        <v>143</v>
+        <v>25</v>
       </c>
       <c r="T4" t="n">
-        <v>87</v>
+        <v>2</v>
       </c>
       <c r="U4" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="V4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W4" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="X4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Z4" t="n">
         <v>0</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF4" t="n">
-        <v>8.473684210526315</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>$81932.46</t>
+          <t>$81554.21</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B5" t="n">
         <v>700000003</v>
@@ -956,11 +952,11 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1021104</v>
+        <v>813431</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CARMENZA RONCANCIO GACHANCIPA</t>
+          <t>Luz Dary Chacon Gaitan</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -969,30 +965,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>7841</v>
+        <v>8425</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>$60143077.08</t>
+          <t>$64916189.91</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>$12312160.00</t>
+          <t>$79769094.00</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>20.47</v>
+        <v>122.88</v>
       </c>
       <c r="M5" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="N5" t="n">
-        <v>33</v>
+        <v>158</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>22.00%</t>
+          <t>106.04%</t>
         </is>
       </c>
       <c r="P5" t="n">
@@ -1002,63 +998,63 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>-9</v>
+        <v>6</v>
       </c>
       <c r="S5" t="n">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="T5" t="n">
-        <v>123</v>
+        <v>45</v>
       </c>
       <c r="U5" t="n">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="V5" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="W5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="X5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Z5" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>14.22%</t>
+          <t>63.71%</t>
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>31</v>
+        <v>139</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>13.36%</t>
+          <t>56.05%</t>
         </is>
       </c>
       <c r="AD5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF5" t="n">
-        <v>8.909090909090908</v>
+        <v>11.63924050632911</v>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>$129277.68</t>
+          <t>$5982682.05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B6" t="n">
         <v>700000003</v>
@@ -1077,11 +1073,11 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>800685</v>
+        <v>1019466</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>JESSICA ROCIO CORTES PERILLA</t>
+          <t>LUZ NANCY ROJAS NEIRA</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1090,7 +1086,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>10168</v>
+        <v>9717</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1099,7 +1095,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>$370613.00</t>
+          <t>$1902444.00</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -1109,36 +1105,36 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S6" t="n">
+        <v>18</v>
+      </c>
+      <c r="T6" t="n">
+        <v>9</v>
+      </c>
+      <c r="U6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S6" t="n">
-        <v>11</v>
-      </c>
-      <c r="T6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X6" t="n">
         <v>0</v>
@@ -1151,15 +1147,15 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>9.09%</t>
+          <t>27.78%</t>
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>22.22%</t>
         </is>
       </c>
       <c r="AD6" t="n">
@@ -1169,17 +1165,17 @@
         <v>0</v>
       </c>
       <c r="AF6" t="n">
-        <v>6</v>
+        <v>10.8</v>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>$5281.24</t>
+          <t>$21402.50</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B7" t="n">
         <v>700000003</v>
@@ -1198,16 +1194,12 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1407710</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>MIGUEL ANGEL MORENO BAUTISTA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>9678</v>
+        <v>9718</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1240,25 +1232,25 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S7" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y7" t="n">
         <v>0</v>
@@ -1268,15 +1260,15 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>18.18%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="AB7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>18.18%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="AD7" t="n">
@@ -1286,7 +1278,7 @@
         <v>0</v>
       </c>
       <c r="AF7" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
@@ -1296,7 +1288,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B8" t="n">
         <v>700000003</v>
@@ -1315,35 +1307,43 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+        <v>985990</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>MARIA CRISTINA RUBIO</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I8" t="n">
-        <v>9718</v>
+        <v>9400</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$17013948.94</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$18007714.00</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>105.84</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>108.77%</t>
         </is>
       </c>
       <c r="P8" t="n">
@@ -1353,63 +1353,63 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="X8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Z8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>63.92%</t>
         </is>
       </c>
       <c r="AB8" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>52.58%</t>
         </is>
       </c>
       <c r="AD8" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
       </c>
       <c r="AF8" t="n">
-        <v>0</v>
+        <v>8.435483870967742</v>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$1089466.70</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B9" t="n">
         <v>700000003</v>
@@ -1428,43 +1428,35 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1077740</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>LUZ MARY LUNA LEON</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>9291</v>
+        <v>8048</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>$31598063.23</t>
+          <t>$000.00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>$6063738.00</t>
+          <t>$000.00</t>
         </is>
       </c>
       <c r="L9" t="n">
-        <v>19.19</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P9" t="n">
@@ -1474,63 +1466,63 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="S9" t="n">
-        <v>135</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="X9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Z9" t="n">
         <v>0</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>11.11%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="AB9" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>10.37%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="AD9" t="n">
         <v>0</v>
       </c>
       <c r="AE9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF9" t="n">
-        <v>8.800000000000001</v>
+        <v>0</v>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>$63669.25</t>
+          <t>$000.00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B10" t="n">
         <v>700000003</v>
@@ -1549,43 +1541,39 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>813431</v>
+        <v>9079</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Luz Dary Chacon Gaitan</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
+          <t>MARIA ELENA PATIÑO FALLA</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>8425</v>
+        <v>9581</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>$77487414.67</t>
+          <t>$000.00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>$22759714.00</t>
+          <t>$000.00</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>29.37</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>152</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>18.42%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P10" t="n">
@@ -1595,43 +1583,43 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>-20</v>
+        <v>-6</v>
       </c>
       <c r="S10" t="n">
-        <v>227</v>
+        <v>18</v>
       </c>
       <c r="T10" t="n">
-        <v>133</v>
+        <v>4</v>
       </c>
       <c r="U10" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="V10" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="W10" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="X10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Y10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Z10" t="n">
         <v>0</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>11.11%</t>
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>11.11%</t>
         </is>
       </c>
       <c r="AD10" t="n">
@@ -1641,17 +1629,17 @@
         <v>0</v>
       </c>
       <c r="AF10" t="n">
-        <v>9.321428571428571</v>
+        <v>10.5</v>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>$238977.00</t>
+          <t>$000.00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B11" t="n">
         <v>700000003</v>
@@ -1670,11 +1658,11 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1297183</v>
+        <v>1741255</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>DORA INES BELTRAN GAMBA</t>
+          <t>EVELYN GOMEZ LOZANO</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1683,7 +1671,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>9948</v>
+        <v>10223</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1692,17 +1680,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$1441718.00</t>
         </is>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1716,63 +1704,63 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>-2</v>
+        <v>3</v>
       </c>
       <c r="S11" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="T11" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="AB11" t="n">
         <v>1</v>
       </c>
-      <c r="W11" t="n">
-        <v>2</v>
-      </c>
-      <c r="X11" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AB11" t="n">
-        <v>0</v>
-      </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>25.00%</t>
         </is>
       </c>
       <c r="AD11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE11" t="n">
         <v>0</v>
       </c>
       <c r="AF11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$22707.06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B12" t="n">
         <v>700000003</v>
@@ -1791,35 +1779,39 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+        <v>768496</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>LUZ ADRIANA PAEZ VIGOYA</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>8048</v>
+        <v>8481</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$56758470.52</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$64954791.00</t>
         </is>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>114.44</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>105.67%</t>
         </is>
       </c>
       <c r="P12" t="n">
@@ -1829,63 +1821,63 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S12" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="V12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="X12" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="Y12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Z12" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>67.73%</t>
         </is>
       </c>
       <c r="AB12" t="n">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>59.55%</t>
         </is>
       </c>
       <c r="AD12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE12" t="n">
         <v>0</v>
       </c>
       <c r="AF12" t="n">
-        <v>0</v>
+        <v>11.87919463087248</v>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$4262658.16</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B13" t="n">
         <v>700000003</v>
@@ -1904,12 +1896,20 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+        <v>800685</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>JESSICA ROCIO CORTES PERILLA</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I13" t="n">
-        <v>10261</v>
+        <v>10168</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$2216237.00</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1928,7 +1928,7 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1942,13 +1942,13 @@
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S13" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1970,35 +1970,35 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="AB13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="AD13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE13" t="n">
         <v>0</v>
       </c>
       <c r="AF13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$36567.91</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B14" t="n">
         <v>700000003</v>
@@ -2022,7 +2022,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>9581</v>
+        <v>9175</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -2055,28 +2055,28 @@
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z14" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B15" t="n">
         <v>700000003</v>
@@ -2130,35 +2130,39 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
+        <v>1099653</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ANGELA MIREYA MONTENEGRO ROMERO</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>9376</v>
+        <v>9334</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$36505654.21</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$39495847.80</t>
         </is>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>108.19</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>106.12%</t>
         </is>
       </c>
       <c r="P15" t="n">
@@ -2168,63 +2172,63 @@
         <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="T15" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="U15" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="V15" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="W15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>67.10%</t>
         </is>
       </c>
       <c r="AB15" t="n">
-        <v>0</v>
+        <v>93</v>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="AD15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF15" t="n">
-        <v>0</v>
+        <v>12.01923076923077</v>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$2280885.21</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B16" t="n">
         <v>700000003</v>
@@ -2243,39 +2247,43 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1019466</v>
+        <v>1021104</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>LUZ NANCY ROJAS NEIRA</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>CARMENZA RONCANCIO GACHANCIPA</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I16" t="n">
-        <v>9717</v>
+        <v>7841</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$48994378.93</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$52140565.00</t>
         </is>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>106.42</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>105.52%</t>
         </is>
       </c>
       <c r="P16" t="n">
@@ -2285,63 +2293,63 @@
         <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S16" t="n">
-        <v>18</v>
+        <v>242</v>
       </c>
       <c r="T16" t="n">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="U16" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="V16" t="n">
+        <v>11</v>
+      </c>
+      <c r="W16" t="n">
+        <v>7</v>
+      </c>
+      <c r="X16" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y16" t="n">
         <v>3</v>
       </c>
-      <c r="W16" t="n">
-        <v>0</v>
-      </c>
-      <c r="X16" t="n">
+      <c r="Z16" t="n">
+        <v>13</v>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>63.22%</t>
+        </is>
+      </c>
+      <c r="AB16" t="n">
+        <v>131</v>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>54.13%</t>
+        </is>
+      </c>
+      <c r="AD16" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE16" t="n">
         <v>3</v>
       </c>
-      <c r="Y16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA16" t="inlineStr">
-        <is>
-          <t>5.56%</t>
-        </is>
-      </c>
-      <c r="AB16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AD16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>0</v>
-      </c>
       <c r="AF16" t="n">
-        <v>5</v>
+        <v>10.59477124183007</v>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$3728050.40</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B17" t="n">
         <v>700000003</v>
@@ -2360,39 +2368,43 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>768496</v>
+        <v>1694138</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>LUZ ADRIANA PAEZ VIGOYA</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
+          <t>YENNY COROMOTO DIAZ PEREZ</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I17" t="n">
-        <v>8481</v>
+        <v>9640</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$63767465.56</t>
+          <t>$000.00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$10739821.00</t>
+          <t>$8597102.00</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>16.84</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>15.44%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P17" t="n">
@@ -2402,63 +2414,63 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>-12</v>
+        <v>6</v>
       </c>
       <c r="S17" t="n">
-        <v>208</v>
+        <v>42</v>
       </c>
       <c r="T17" t="n">
-        <v>133</v>
+        <v>4</v>
       </c>
       <c r="U17" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="V17" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="W17" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="X17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Y17" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="Z17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>10.10%</t>
+          <t>73.81%</t>
         </is>
       </c>
       <c r="AB17" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>10.10%</t>
+          <t>52.38%</t>
         </is>
       </c>
       <c r="AD17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE17" t="n">
         <v>0</v>
       </c>
       <c r="AF17" t="n">
-        <v>10.71428571428571</v>
+        <v>8.451612903225806</v>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>$112768.12</t>
+          <t>$154747.84</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B18" t="n">
         <v>700000003</v>
@@ -2477,12 +2489,20 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+        <v>1407710</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>MIGUEL ANGEL MORENO BAUTISTA</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I18" t="n">
-        <v>10255</v>
+        <v>9678</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -2491,7 +2511,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$1422374.00</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -2501,7 +2521,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2515,43 +2535,43 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S18" t="n">
+        <v>11</v>
+      </c>
+      <c r="T18" t="n">
+        <v>4</v>
+      </c>
+      <c r="U18" t="n">
+        <v>2</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" t="n">
         <v>1</v>
       </c>
-      <c r="T18" t="n">
+      <c r="X18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" t="n">
         <v>1</v>
       </c>
-      <c r="U18" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" t="n">
-        <v>0</v>
-      </c>
-      <c r="W18" t="n">
-        <v>0</v>
-      </c>
-      <c r="X18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>0</v>
-      </c>
       <c r="Z18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>45.45%</t>
         </is>
       </c>
       <c r="AB18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>36.36%</t>
         </is>
       </c>
       <c r="AD18" t="n">
@@ -2561,17 +2581,17 @@
         <v>0</v>
       </c>
       <c r="AF18" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$17068.49</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>202612</v>
+        <v>202611</v>
       </c>
       <c r="B19" t="n">
         <v>700000003</v>
@@ -2590,11 +2610,11 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1741255</v>
+        <v>1077740</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>EVELYN GOMEZ LOZANO</t>
+          <t>LUZ MARY LUNA LEON</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2603,30 +2623,30 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>10223</v>
+        <v>9291</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$26606005.43</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>$000.00</t>
+          <t>$27489699.00</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>103.32</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>106.82%</t>
         </is>
       </c>
       <c r="P19" t="n">
@@ -2639,296 +2659,54 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>4</v>
+        <v>141</v>
       </c>
       <c r="T19" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="U19" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="V19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W19" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Z19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>66.67%</t>
         </is>
       </c>
       <c r="AB19" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>56.03%</t>
         </is>
       </c>
       <c r="AD19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AF19" t="n">
-        <v>0</v>
+        <v>8.595744680851064</v>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>$000.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B20" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>1665372</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>DORIS ANGARITA</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>10260</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>$000.00</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>$000.00</t>
-        </is>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" t="n">
-        <v>1</v>
-      </c>
-      <c r="T20" t="n">
-        <v>1</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="n">
-        <v>0</v>
-      </c>
-      <c r="W20" t="n">
-        <v>0</v>
-      </c>
-      <c r="X20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AB20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC20" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AD20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG20" t="inlineStr">
-        <is>
-          <t>$000.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B21" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>985990</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>MARIA CRISTINA RUBIO</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>9400</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>$23747542.18</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>$1573859.00</t>
-        </is>
-      </c>
-      <c r="L21" t="n">
-        <v>6.63</v>
-      </c>
-      <c r="M21" t="n">
-        <v>68</v>
-      </c>
-      <c r="N21" t="n">
-        <v>5</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>7.35%</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" t="n">
-        <v>-11</v>
-      </c>
-      <c r="S21" t="n">
-        <v>94</v>
-      </c>
-      <c r="T21" t="n">
-        <v>59</v>
-      </c>
-      <c r="U21" t="n">
-        <v>17</v>
-      </c>
-      <c r="V21" t="n">
-        <v>13</v>
-      </c>
-      <c r="W21" t="n">
-        <v>12</v>
-      </c>
-      <c r="X21" t="n">
-        <v>10</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>9</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>5.32%</t>
-        </is>
-      </c>
-      <c r="AB21" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC21" t="inlineStr">
-        <is>
-          <t>5.32%</t>
-        </is>
-      </c>
-      <c r="AD21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF21" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG21" t="inlineStr">
-        <is>
-          <t>$16525.52</t>
+          <t>$1285143.43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar bases de datos y mapeos json de objetivos arte y usuarios
</commit_message>
<xml_diff>
--- a/Base para el como vamos.xlsx
+++ b/Base para el como vamos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Base para el como vamos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Como vamos anterior" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base para el como vamos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Como vamos anterior" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>$4159446.00</t>
+          <t>$6130751.00</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -750,11 +750,11 @@
         <v>29</v>
       </c>
       <c r="N3" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>44.83%</t>
+          <t>75.86%</t>
         </is>
       </c>
       <c r="P3" t="n">
@@ -764,13 +764,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="T3" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="U3" t="n">
         <v>4</v>
@@ -792,29 +792,29 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>31.71%</t>
+          <t>52.38%</t>
         </is>
       </c>
       <c r="AB3" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>26.83%</t>
+          <t>45.24%</t>
         </is>
       </c>
       <c r="AD3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>8.76923076923077</v>
+        <v>7.681818181818182</v>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>$49913.35</t>
+          <t>$78167.08</t>
         </is>
       </c>
     </row>
@@ -857,21 +857,21 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>$34105248.00</t>
+          <t>$40723054.00</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>83.39</v>
+        <v>99.56999999999999</v>
       </c>
       <c r="M4" t="n">
         <v>96</v>
       </c>
       <c r="N4" t="n">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>79.17%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="P4" t="n">
@@ -881,22 +881,22 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="S4" t="n">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="T4" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="U4" t="n">
         <v>21</v>
       </c>
       <c r="V4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X4" t="n">
         <v>5</v>
@@ -905,33 +905,33 @@
         <v>5</v>
       </c>
       <c r="Z4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>50.67%</t>
+          <t>62.75%</t>
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>46.00%</t>
+          <t>56.21%</t>
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>9.934210526315789</v>
+        <v>9.427083333333334</v>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>$358105.10</t>
+          <t>$1058799.40</t>
         </is>
       </c>
     </row>
@@ -978,21 +978,21 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>$48505978.00</t>
+          <t>$53822764.00</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>83.56</v>
+        <v>92.72</v>
       </c>
       <c r="M5" t="n">
         <v>150</v>
       </c>
       <c r="N5" t="n">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>82.00%</t>
+          <t>96.00%</t>
         </is>
       </c>
       <c r="P5" t="n">
@@ -1002,22 +1002,22 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="S5" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="T5" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="U5" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="V5" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="W5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="X5" t="n">
         <v>6</v>
@@ -1026,19 +1026,19 @@
         <v>4</v>
       </c>
       <c r="Z5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>52.34%</t>
+          <t>61.02%</t>
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>50.21%</t>
+          <t>58.47%</t>
         </is>
       </c>
       <c r="AD5" t="n">
@@ -1048,11 +1048,11 @@
         <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>10.11382113821138</v>
+        <v>9.701388888888889</v>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>$509312.77</t>
+          <t>$602814.96</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>$2698136.00</t>
+          <t>$3835572.00</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -1109,7 +1109,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1123,13 +1123,13 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="T6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U6" t="n">
         <v>2</v>
@@ -1151,29 +1151,29 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>60.00%</t>
+          <t>76.47%</t>
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>26.67%</t>
+          <t>35.29%</t>
         </is>
       </c>
       <c r="AD6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
       </c>
       <c r="AF6" t="n">
-        <v>8</v>
+        <v>8.23076923076923</v>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>$46542.85</t>
+          <t>$69040.30</t>
         </is>
       </c>
     </row>
@@ -1450,21 +1450,21 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>$22431333.00</t>
+          <t>$25662444.00</t>
         </is>
       </c>
       <c r="L9" t="n">
-        <v>73.43000000000001</v>
+        <v>84</v>
       </c>
       <c r="M9" t="n">
         <v>87</v>
       </c>
       <c r="N9" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>75.86%</t>
+          <t>88.51%</t>
         </is>
       </c>
       <c r="P9" t="n">
@@ -1474,43 +1474,43 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S9" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="T9" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="U9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="V9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X9" t="n">
         <v>7</v>
       </c>
       <c r="Y9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>46.48%</t>
+          <t>53.47%</t>
         </is>
       </c>
       <c r="AB9" t="n">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>41.55%</t>
+          <t>47.22%</t>
         </is>
       </c>
       <c r="AD9" t="n">
@@ -1520,11 +1520,11 @@
         <v>2</v>
       </c>
       <c r="AF9" t="n">
-        <v>7.833333333333333</v>
+        <v>7.662337662337662</v>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>$336470.00</t>
+          <t>$423430.33</t>
         </is>
       </c>
     </row>
@@ -1571,21 +1571,21 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>$63384447.00</t>
+          <t>$73520285.00</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>85.95999999999999</v>
+        <v>99.70999999999999</v>
       </c>
       <c r="M10" t="n">
         <v>152</v>
       </c>
       <c r="N10" t="n">
-        <v>118</v>
+        <v>145</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>77.63%</t>
+          <t>95.39%</t>
         </is>
       </c>
       <c r="P10" t="n">
@@ -1595,22 +1595,22 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="S10" t="n">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="T10" t="n">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="U10" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="V10" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="W10" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="X10" t="n">
         <v>5</v>
@@ -1619,33 +1619,33 @@
         <v>7</v>
       </c>
       <c r="Z10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>60.67%</t>
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>46.19%</t>
+          <t>55.65%</t>
         </is>
       </c>
       <c r="AD10" t="n">
         <v>1</v>
       </c>
       <c r="AE10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF10" t="n">
-        <v>10.16949152542373</v>
+        <v>10.0551724137931</v>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>$665536.69</t>
+          <t>$1415265.49</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>$3037831.00</t>
+          <t>$4239786.00</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1702,11 +1702,11 @@
         <v>19</v>
       </c>
       <c r="N11" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>42.11%</t>
+          <t>73.68%</t>
         </is>
       </c>
       <c r="P11" t="n">
@@ -1716,13 +1716,13 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="T11" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="U11" t="n">
         <v>2</v>
@@ -1744,29 +1744,29 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>53.85%</t>
         </is>
       </c>
       <c r="AB11" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>29.17%</t>
+          <t>42.31%</t>
         </is>
       </c>
       <c r="AD11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE11" t="n">
         <v>0</v>
       </c>
       <c r="AF11" t="n">
-        <v>11.875</v>
+        <v>8.928571428571429</v>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>$36453.97</t>
+          <t>$60416.95</t>
         </is>
       </c>
     </row>
@@ -2378,21 +2378,21 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>$51084500.01</t>
+          <t>$58404352.01</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>84.36</v>
+        <v>96.45</v>
       </c>
       <c r="M17" t="n">
         <v>136</v>
       </c>
       <c r="N17" t="n">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>76.47%</t>
+          <t>88.97%</t>
         </is>
       </c>
       <c r="P17" t="n">
@@ -2402,22 +2402,22 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="S17" t="n">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="T17" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="U17" t="n">
         <v>27</v>
       </c>
       <c r="V17" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="W17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="X17" t="n">
         <v>8</v>
@@ -2426,33 +2426,33 @@
         <v>12</v>
       </c>
       <c r="Z17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>48.60%</t>
+          <t>56.02%</t>
         </is>
       </c>
       <c r="AB17" t="n">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>45.79%</t>
+          <t>52.31%</t>
         </is>
       </c>
       <c r="AD17" t="n">
         <v>2</v>
       </c>
       <c r="AE17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF17" t="n">
-        <v>10.65384615384615</v>
+        <v>10.80165289256198</v>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>$536387.25</t>
+          <t>$654128.74</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>$1866132.00</t>
+          <t>$2238902.00</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -2626,7 +2626,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2640,10 +2640,10 @@
         <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T19" t="n">
         <v>1</v>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>83.33%</t>
+          <t>85.71%</t>
         </is>
       </c>
       <c r="AB19" t="n">
@@ -2676,21 +2676,21 @@
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>42.86%</t>
         </is>
       </c>
       <c r="AD19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE19" t="n">
         <v>0</v>
       </c>
       <c r="AF19" t="n">
-        <v>9.4</v>
+        <v>9.666666666666666</v>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>$27991.98</t>
+          <t>$35262.71</t>
         </is>
       </c>
     </row>
@@ -2858,21 +2858,21 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>$12760156.00</t>
+          <t>$14368309.00</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>56.67</v>
+        <v>63.81</v>
       </c>
       <c r="M21" t="n">
         <v>68</v>
       </c>
       <c r="N21" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>60.29%</t>
+          <t>72.06%</t>
         </is>
       </c>
       <c r="P21" t="n">
@@ -2882,13 +2882,13 @@
         <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="S21" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="T21" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="U21" t="n">
         <v>16</v>
@@ -2897,42 +2897,42 @@
         <v>12</v>
       </c>
       <c r="W21" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="X21" t="n">
         <v>10</v>
       </c>
       <c r="Y21" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>41.41%</t>
+          <t>47.12%</t>
         </is>
       </c>
       <c r="AB21" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>36.36%</t>
+          <t>37.50%</t>
         </is>
       </c>
       <c r="AD21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF21" t="n">
-        <v>7.951219512195122</v>
+        <v>7.469387755102041</v>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>$133981.64</t>
+          <t>$172419.71</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: banner ejecutivo de cartera pendiente con cruce de vencimientos GERA, calibracion de paleta de colores y pasarela Evolution API
</commit_message>
<xml_diff>
--- a/Base para el como vamos.xlsx
+++ b/Base para el como vamos.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG21"/>
+  <dimension ref="A1:AG41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2933,6 +2933,2334 @@
       <c r="AG21" t="inlineStr">
         <is>
           <t>$172419.71</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B22" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>162200</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>JUANA MARCELA LINARES CARDENAS</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>9337</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>2200558</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>4</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-6</v>
+      </c>
+      <c r="S22" t="n">
+        <v>42</v>
+      </c>
+      <c r="T22" t="n">
+        <v>26</v>
+      </c>
+      <c r="U22" t="n">
+        <v>10</v>
+      </c>
+      <c r="V22" t="n">
+        <v>2</v>
+      </c>
+      <c r="W22" t="n">
+        <v>6</v>
+      </c>
+      <c r="X22" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>9.52%</t>
+        </is>
+      </c>
+      <c r="AB22" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>9.52%</t>
+        </is>
+      </c>
+      <c r="AD22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B23" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>262044</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>YADIRA MARIA CORREALES ROJAS</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>9924</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>728422</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>2</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S23" t="n">
+        <v>38</v>
+      </c>
+      <c r="T23" t="n">
+        <v>28</v>
+      </c>
+      <c r="U23" t="n">
+        <v>3</v>
+      </c>
+      <c r="V23" t="n">
+        <v>5</v>
+      </c>
+      <c r="W23" t="n">
+        <v>4</v>
+      </c>
+      <c r="X23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>5.26%</t>
+        </is>
+      </c>
+      <c r="AB23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>5.26%</t>
+        </is>
+      </c>
+      <c r="AD23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B24" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1082490</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ROSA REINALDA PINILLA VELASQUEZ</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>7817</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>$40729756.27</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>$6620104.00</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="M24" t="n">
+        <v>111</v>
+      </c>
+      <c r="N24" t="n">
+        <v>18</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>16.22%</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="n">
+        <v>-16</v>
+      </c>
+      <c r="S24" t="n">
+        <v>155</v>
+      </c>
+      <c r="T24" t="n">
+        <v>70</v>
+      </c>
+      <c r="U24" t="n">
+        <v>45</v>
+      </c>
+      <c r="V24" t="n">
+        <v>22</v>
+      </c>
+      <c r="W24" t="n">
+        <v>16</v>
+      </c>
+      <c r="X24" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>11</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>11.61%</t>
+        </is>
+      </c>
+      <c r="AB24" t="n">
+        <v>18</v>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>11.61%</t>
+        </is>
+      </c>
+      <c r="AD24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>9.166666666666666</v>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>$69511.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B25" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>9405</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B26" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1037030</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>DIANA PATRICIA APARICIO AVILA</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="n">
+        <v>9529</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>$42993213.16</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>$9324859.00</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>21.69</v>
+      </c>
+      <c r="M26" t="n">
+        <v>91</v>
+      </c>
+      <c r="N26" t="n">
+        <v>16</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>17.58%</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" t="n">
+        <v>-11</v>
+      </c>
+      <c r="S26" t="n">
+        <v>129</v>
+      </c>
+      <c r="T26" t="n">
+        <v>68</v>
+      </c>
+      <c r="U26" t="n">
+        <v>31</v>
+      </c>
+      <c r="V26" t="n">
+        <v>14</v>
+      </c>
+      <c r="W26" t="n">
+        <v>11</v>
+      </c>
+      <c r="X26" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>12.40%</t>
+        </is>
+      </c>
+      <c r="AB26" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>11.63%</t>
+        </is>
+      </c>
+      <c r="AD26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>14.8125</v>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>$97911.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B27" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>13774</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>JACKELINE OSMA VARGAS</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>5060</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>$63154330.43</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>$13141897.00</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>20.81</v>
+      </c>
+      <c r="M27" t="n">
+        <v>146</v>
+      </c>
+      <c r="N27" t="n">
+        <v>23</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>15.75%</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="n">
+        <v>-8</v>
+      </c>
+      <c r="S27" t="n">
+        <v>218</v>
+      </c>
+      <c r="T27" t="n">
+        <v>128</v>
+      </c>
+      <c r="U27" t="n">
+        <v>36</v>
+      </c>
+      <c r="V27" t="n">
+        <v>31</v>
+      </c>
+      <c r="W27" t="n">
+        <v>8</v>
+      </c>
+      <c r="X27" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>10.55%</t>
+        </is>
+      </c>
+      <c r="AB27" t="n">
+        <v>22</v>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>10.09%</t>
+        </is>
+      </c>
+      <c r="AD27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>10.21739130434783</v>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>$137989.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B28" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1038108</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>DAAISY CATALINA VIANCHA MERCHAN</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>10293</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>826701</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>2</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="n">
+        <v>2</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="AB28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="AD28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>11</v>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B29" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="n">
+        <v>8055</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" t="n">
+        <v>0</v>
+      </c>
+      <c r="U29" t="n">
+        <v>0</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" t="n">
+        <v>1</v>
+      </c>
+      <c r="X29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AD29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B30" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>5735</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AD30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B31" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="n">
+        <v>8928</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B32" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1714795</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>DERLY VIVIANA SOLANO MARIÑO</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="n">
+        <v>10215</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>$42898429.68</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>$12083536.00</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>28.17</v>
+      </c>
+      <c r="M32" t="n">
+        <v>100</v>
+      </c>
+      <c r="N32" t="n">
+        <v>16</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>16.00%</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S32" t="n">
+        <v>157</v>
+      </c>
+      <c r="T32" t="n">
+        <v>97</v>
+      </c>
+      <c r="U32" t="n">
+        <v>30</v>
+      </c>
+      <c r="V32" t="n">
+        <v>14</v>
+      </c>
+      <c r="W32" t="n">
+        <v>4</v>
+      </c>
+      <c r="X32" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>10.19%</t>
+        </is>
+      </c>
+      <c r="AB32" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>9.55%</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>13.9375</v>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>$126877.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B33" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1653163</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>PATRICIA PADILLA RODRÍGUEZ</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="n">
+        <v>10066</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>746938</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>2</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S33" t="n">
+        <v>12</v>
+      </c>
+      <c r="T33" t="n">
+        <v>7</v>
+      </c>
+      <c r="U33" t="n">
+        <v>2</v>
+      </c>
+      <c r="V33" t="n">
+        <v>1</v>
+      </c>
+      <c r="W33" t="n">
+        <v>1</v>
+      </c>
+      <c r="X33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="AB33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="AD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>11</v>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B34" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="n">
+        <v>9591</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B35" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>313643</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>NORMA LUCIA GARZON CASALLAS</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>9891</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>2881675</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>5</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S35" t="n">
+        <v>36</v>
+      </c>
+      <c r="T35" t="n">
+        <v>15</v>
+      </c>
+      <c r="U35" t="n">
+        <v>9</v>
+      </c>
+      <c r="V35" t="n">
+        <v>7</v>
+      </c>
+      <c r="W35" t="n">
+        <v>2</v>
+      </c>
+      <c r="X35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>13.89%</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>11.11%</t>
+        </is>
+      </c>
+      <c r="AD35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B36" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="n">
+        <v>9882</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AD36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B37" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>14107</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>DIANA LUZ AVELLA PINTO</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="n">
+        <v>177</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>$89903621.08</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>$25266929.50</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="M37" t="n">
+        <v>186</v>
+      </c>
+      <c r="N37" t="n">
+        <v>35</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>18.82%</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>-10</v>
+      </c>
+      <c r="S37" t="n">
+        <v>279</v>
+      </c>
+      <c r="T37" t="n">
+        <v>150</v>
+      </c>
+      <c r="U37" t="n">
+        <v>61</v>
+      </c>
+      <c r="V37" t="n">
+        <v>33</v>
+      </c>
+      <c r="W37" t="n">
+        <v>10</v>
+      </c>
+      <c r="X37" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>12.54%</t>
+        </is>
+      </c>
+      <c r="AB37" t="n">
+        <v>33</v>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>11.83%</t>
+        </is>
+      </c>
+      <c r="AD37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>16.14285714285714</v>
+      </c>
+      <c r="AG37" t="inlineStr">
+        <is>
+          <t>$265302.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B38" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>194242</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>ALIX PATRICIA CAMARGO HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="n">
+        <v>9349</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>$43117320.71</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>$7580443.00</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
+        <v>17.58</v>
+      </c>
+      <c r="M38" t="n">
+        <v>107</v>
+      </c>
+      <c r="N38" t="n">
+        <v>19</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>17.76%</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" t="n">
+        <v>-8</v>
+      </c>
+      <c r="S38" t="n">
+        <v>155</v>
+      </c>
+      <c r="T38" t="n">
+        <v>77</v>
+      </c>
+      <c r="U38" t="n">
+        <v>41</v>
+      </c>
+      <c r="V38" t="n">
+        <v>18</v>
+      </c>
+      <c r="W38" t="n">
+        <v>10</v>
+      </c>
+      <c r="X38" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>12.26%</t>
+        </is>
+      </c>
+      <c r="AB38" t="n">
+        <v>17</v>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>10.97%</t>
+        </is>
+      </c>
+      <c r="AD38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>10.10526315789474</v>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>$79594.65</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B39" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="n">
+        <v>7796</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AB39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AD39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B40" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1645714</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>LAURA CATALINA HERNANDEZ PEÑALOZA</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="n">
+        <v>10294</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>294150</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" t="n">
+        <v>1</v>
+      </c>
+      <c r="T40" t="n">
+        <v>0</v>
+      </c>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" t="n">
+        <v>0</v>
+      </c>
+      <c r="W40" t="n">
+        <v>0</v>
+      </c>
+      <c r="X40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="AB40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="AD40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>15</v>
+      </c>
+      <c r="AG40" t="inlineStr">
+        <is>
+          <t>$000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>202613</v>
+      </c>
+      <c r="B41" t="n">
+        <v>700000003</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>GERENCIA VENTAS ARTE KARENTH</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>700000466</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTOR EMOCIONES DOLLY  </t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1101830</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>ESPERANZA CARDENAS BELLO</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>7815</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>$45350720.44</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>$5523409.00</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="M41" t="n">
+        <v>122</v>
+      </c>
+      <c r="N41" t="n">
+        <v>10</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>8.20%</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" t="n">
+        <v>-18</v>
+      </c>
+      <c r="S41" t="n">
+        <v>175</v>
+      </c>
+      <c r="T41" t="n">
+        <v>104</v>
+      </c>
+      <c r="U41" t="n">
+        <v>35</v>
+      </c>
+      <c r="V41" t="n">
+        <v>26</v>
+      </c>
+      <c r="W41" t="n">
+        <v>18</v>
+      </c>
+      <c r="X41" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>5.71%</t>
+        </is>
+      </c>
+      <c r="AB41" t="n">
+        <v>9</v>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>5.14%</t>
+        </is>
+      </c>
+      <c r="AD41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>$57995.79</t>
         </is>
       </c>
     </row>

</xml_diff>